<commit_message>
ORFS: forged face-seal legs at every measured size; no-step / raised-neck masters
- fsmeasure: the forged run-out variants step_up (FS6500-06 / -10, FS2501-08-08-FG) and none
  (FS6500-04 / -12 / -16); pilots revalidated, 0 FAIL, readings unchanged
- gen_straight2: FSMF_MEAS (forged legs -04 ... -20 from FS6500-NN), FSM_MEAS -24 / -32
  (FS2403-24-24, FS6400-32-32-O)
- gen_tee: step up allowed; legs with flats = thread (no step) and adjustable studs whose neck
  lies below the flats get their own masters (<root>N / R / NR, one sketch per master); the
  no-step hex arm ends at the thread end
- 62 FS configurations in the forged + straight closed loops, 1,572 checks, 0 off; the new
  hex-over-thread check proven on the unfixed arm; regression 99 / 99 identical

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQuceHR8ZUuy6411Z8yX1P
</commit_message>
<xml_diff>
--- a/tools/_out/orfs_gen_20261020/out/DesignTable_FS2403_SW2.xlsx
+++ b/tools/_out/orfs_gen_20261020/out/DesignTable_FS2403_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AU3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,6 +808,169 @@
       <c r="AU2" t="inlineStr">
         <is>
           <t>FS2403-08-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FS2403-24-24</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.22976</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.8145</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="I3" t="n">
+        <v>45</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.4676</v>
+      </c>
+      <c r="L3" t="n">
+        <v>60</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.9405</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.12505</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.5296</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.8145</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.4676</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0.9405</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.12505</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0.5296</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>0.04511</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>0.02083</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>FS2403-24-24</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>ORFS Male Union (male face seal x male face seal), 2-12 UN (male O-ring face seal, SAE J1453) x 2-12 UN (male O-ring face seal, SAE J1453)</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>FS2403</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>2-12 UN (male O-ring face seal, SAE J1453)</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>2-12 UN (male O-ring face seal, SAE J1453)</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>Air-Way FF2403 (s9, double-pass 2026-10-15, parts.air-way.com/api/series/9, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p3 FS2403-24-24 (ORFS-p003-t03) | MODEL: L6 face -&gt; face, hex S1, bores D1 (both sides): review table (Air-Way, staged FS table; OMi website list decides the parts); hex over the whole length between the two ends; bore step at the hex mid-plane (ASSUMPTION, as 2403; no effect where the two bores are equal); hex end chamfers NOT modelled; male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-24-24 (both ends; fsmeasure.measure_fsm, orfs_steps2_20261020 ends_survey); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part); male O-ring face-seal end (SAE J1453): thread = the face-seal thread of the dash (Air-Way callout = Brennan ORFS catalog); face O-ring groove (inner / outer dia, depth), land, 45deg nose chamfer, thread length, 60deg flank, relief and end length measured on the Brennan pilot of that dash (Brennan FS2403-24-24 (both ends; fsmeasure.measure_fsm, orfs_steps2_20261020 ends_survey); single manufacturer - Air-Way 3D models not yet measured, Q-FS-2NDSHAPE); groove drawn rectangular (its outer bottom corner is hidden under the O-ring Brennan fuses into the solid - ASSUMPTION); O-ring not modelled (separate FS4000 part)</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>Air-Way FF2403 = Brennan p3 on overall length, hex (rounding-only differences count as equal) | OMi parts file row 5273 (no dimensions) | DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>FS2403-24-24</t>
         </is>
       </c>
     </row>

</xml_diff>